<commit_message>
20260501_172202 - baseline with April 26 src + April 28/29 updates, camera working
</commit_message>
<xml_diff>
--- a/app/src/main/assets/templates/elevator_monthly_report.xlsx
+++ b/app/src/main/assets/templates/elevator_monthly_report.xlsx
@@ -4,7 +4,7 @@
   <fileVersion appName="xl" lastEdited="3" lowestEdited="5" rupBuild="9302"/>
   <workbookPr codeName="ThisWorkbook"/>
   <bookViews>
-    <workbookView windowWidth="29868" windowHeight="12935" activeTab="1"/>
+    <workbookView windowWidth="30720" windowHeight="12935"/>
   </bookViews>
   <sheets>
     <sheet name="办公楼报告" sheetId="112" r:id="rId1"/>
@@ -14,7 +14,7 @@
     <definedName name="_xlnm.Print_Area" localSheetId="0">办公楼报告!$A$1:$R$48</definedName>
     <definedName name="_xlnm.Print_Area" localSheetId="1">商场报告!$A$1:$V$83</definedName>
   </definedNames>
-  <calcPr calcId="191029" fullCalcOnLoad="1"/>
+  <calcPr calcId="191029"/>
   <customWorkbookViews>
     <customWorkbookView name="kymtang - 个人视图" guid="{B9BA8337-1B7F-4DB2-BC23-2E5B288FACA4}" personalView="1" maximized="1" windowWidth="1276" windowHeight="781" activeSheetId="0"/>
   </customWorkbookViews>
@@ -328,7 +328,12 @@
     <numFmt numFmtId="44" formatCode="_ &quot;￥&quot;* #,##0.00_ ;_ &quot;￥&quot;* \-#,##0.00_ ;_ &quot;￥&quot;* &quot;-&quot;??_ ;_ @_ "/>
     <numFmt numFmtId="176" formatCode="0.00_ "/>
   </numFmts>
-  <fonts count="29">
+  <fonts count="31">
+    <font>
+      <sz val="12"/>
+      <name val="宋体"/>
+      <charset val="134"/>
+    </font>
     <font>
       <sz val="12"/>
       <name val="宋体"/>
@@ -522,6 +527,13 @@
       <sz val="10"/>
       <name val="Arial"/>
       <charset val="134"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="宋体"/>
+      <charset val="134"/>
+      <scheme val="minor"/>
     </font>
     <font>
       <sz val="10"/>
@@ -1102,371 +1114,371 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="43" fontId="7" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="44" fontId="7" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="9" fontId="7" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="41" fontId="7" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="42" fontId="7" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="43" fontId="8" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="44" fontId="8" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="9" fontId="8" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="41" fontId="8" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="42" fontId="8" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="2" borderId="23" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="10" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="8" fillId="2" borderId="23" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="11" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="12" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="24" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="14" fillId="0" borderId="24" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="25" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="3" borderId="26" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="4" borderId="27" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="4" borderId="26" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="5" borderId="28" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="0" borderId="29" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="0" borderId="30" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="6" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="7" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="8" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="25" fillId="9" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="26" fillId="10" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="26" fillId="11" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="25" fillId="12" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="25" fillId="13" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="26" fillId="14" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="26" fillId="15" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="25" fillId="16" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="25" fillId="17" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="26" fillId="18" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="26" fillId="19" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="25" fillId="20" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="25" fillId="21" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="26" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="26" fillId="23" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="25" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="25" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="26" fillId="26" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="26" fillId="27" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="25" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="25" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="26" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="26" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="25" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="27" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="27" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0">
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="24" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="25" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="3" borderId="26" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="4" borderId="27" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="4" borderId="26" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="5" borderId="28" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="0" borderId="29" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="0" borderId="30" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="6" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="7" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="8" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="26" fillId="9" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="27" fillId="10" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="27" fillId="11" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="26" fillId="12" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="26" fillId="13" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="27" fillId="14" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="27" fillId="15" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="26" fillId="16" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="26" fillId="17" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="27" fillId="18" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="27" fillId="19" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="26" fillId="20" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="26" fillId="21" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="27" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="27" fillId="23" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="26" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="26" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="27" fillId="26" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="27" fillId="27" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="26" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="26" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="27" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="27" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="26" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="28" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="29" fillId="0" borderId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="29" fillId="0" borderId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="29" fillId="0" borderId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="29" fillId="0" borderId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="29" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="29" fillId="0" borderId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="29" fillId="0" borderId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="28" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="29" fillId="0" borderId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="29" fillId="0" borderId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="30" fillId="0" borderId="0"/>
   </cellStyleXfs>
   <cellXfs count="53">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="78">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="78" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="78">
+      <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="78" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="78" applyFont="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="78" applyAlignment="1">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="78" applyBorder="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="2" xfId="78" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="3" xfId="78" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="4" xfId="78" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="5" xfId="78" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="6" xfId="78" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="7" xfId="78" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="8" xfId="78" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="78" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="9" xfId="78" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="78" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="11" xfId="78" applyFont="1" applyBorder="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="12" xfId="78" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="13" xfId="78" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="11" xfId="78" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="12" xfId="78" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="13" xfId="78" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="78" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="14" xfId="78" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="15" xfId="78" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="16" xfId="78" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="17" xfId="78" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="78" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="18" xfId="78" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="78" applyFont="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="78" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="78" applyBorder="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="2" xfId="78" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="3" xfId="78" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="19" xfId="78" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="4" xfId="78" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="12" xfId="78" applyBorder="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="20" xfId="78" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="5" xfId="78" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="21" xfId="78" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="6" xfId="78" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="176" fontId="3" fillId="0" borderId="1" xfId="78" applyNumberFormat="1" applyFont="1" applyBorder="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="78" applyFont="1" applyBorder="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="78" applyFont="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="78" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="7" xfId="78" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="8" xfId="78" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="78" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="9" xfId="78" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="10" xfId="78" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="11" xfId="78" applyFont="1" applyBorder="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="12" xfId="78" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="13" xfId="78" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="11" xfId="78" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="12" xfId="78" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="78" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="12" xfId="78" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="14" xfId="78" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="15" xfId="78" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="16" xfId="78" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="17" xfId="78" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="78" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="18" xfId="78" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="19" xfId="78" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="12" xfId="78" applyBorder="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="20" xfId="78" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="21" xfId="78" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="176" fontId="4" fillId="0" borderId="1" xfId="78" applyNumberFormat="1" applyFont="1" applyBorder="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="78" applyFont="1" applyBorder="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="78" applyFont="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="78" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="78" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="78" applyFont="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="78" applyFont="1" applyBorder="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="78" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="1" xfId="78" applyFont="1" applyBorder="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="1" xfId="78" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="78" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="78" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="14" fontId="6" fillId="0" borderId="22" xfId="78" applyNumberFormat="1" applyFont="1" applyBorder="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="14" fontId="6" fillId="0" borderId="0" xfId="78" applyNumberFormat="1" applyFont="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="14" fontId="6" fillId="0" borderId="22" xfId="78" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="14" fontId="7" fillId="0" borderId="22" xfId="78" applyNumberFormat="1" applyFont="1" applyBorder="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="14" fontId="7" fillId="0" borderId="0" xfId="78" applyNumberFormat="1" applyFont="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="14" fontId="7" fillId="0" borderId="22" xfId="78" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="22" xfId="78" applyBorder="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="22" xfId="78" applyFont="1" applyBorder="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="22" xfId="78" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="22" xfId="78" applyBorder="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="22" xfId="78" applyFont="1" applyBorder="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="22" xfId="78" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="78" applyFont="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="13" xfId="78" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="13" xfId="78" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="13" xfId="78" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="15" xfId="78" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="78" applyFont="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="13" xfId="78" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="13" xfId="78" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="13" xfId="78" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="15" xfId="78" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="80">
@@ -2309,7 +2321,7 @@
       <c r="O11" s="21"/>
       <c r="P11" s="21"/>
       <c r="Q11" s="21"/>
-      <c r="R11" s="22"/>
+      <c r="R11" s="19"/>
     </row>
     <row r="12" ht="11.1" customHeight="1" spans="1:19">
       <c r="A12" s="20">
@@ -2331,7 +2343,7 @@
       <c r="O12" s="21"/>
       <c r="P12" s="21"/>
       <c r="Q12" s="21"/>
-      <c r="R12" s="22"/>
+      <c r="R12" s="19"/>
     </row>
     <row r="13" ht="11.1" customHeight="1" spans="1:19">
       <c r="A13" s="20">
@@ -2513,7 +2525,7 @@
       <c r="A21" s="20">
         <v>14</v>
       </c>
-      <c r="B21" s="23"/>
+      <c r="B21" s="22"/>
       <c r="C21" s="21"/>
       <c r="D21" s="21"/>
       <c r="E21" s="21"/>
@@ -2525,7 +2537,7 @@
       <c r="K21" s="21"/>
       <c r="L21" s="21"/>
       <c r="M21" s="21"/>
-      <c r="N21" s="21"/>
+      <c r="N21" s="23"/>
       <c r="O21" s="21"/>
       <c r="P21" s="21"/>
       <c r="Q21" s="21"/>
@@ -2595,7 +2607,7 @@
       <c r="O24" s="21"/>
       <c r="P24" s="21"/>
       <c r="Q24" s="21"/>
-      <c r="R24" s="22"/>
+      <c r="R24" s="19"/>
     </row>
     <row r="25" ht="11.1" customHeight="1" spans="1:18">
       <c r="A25" s="20">
@@ -2771,7 +2783,7 @@
       <c r="O32" s="21"/>
       <c r="P32" s="21"/>
       <c r="Q32" s="21"/>
-      <c r="R32" s="22"/>
+      <c r="R32" s="19"/>
     </row>
     <row r="33" ht="11.1" customHeight="1" spans="1:21">
       <c r="A33" s="20">
@@ -3359,7 +3371,7 @@
       <c r="S8" s="21"/>
       <c r="T8" s="21"/>
       <c r="U8" s="21"/>
-      <c r="V8" s="22"/>
+      <c r="V8" s="19"/>
     </row>
     <row r="9" ht="11.1" customHeight="1" spans="1:23">
       <c r="A9" s="20">
@@ -3385,7 +3397,7 @@
       <c r="S9" s="21"/>
       <c r="T9" s="21"/>
       <c r="U9" s="21"/>
-      <c r="V9" s="22"/>
+      <c r="V9" s="19"/>
     </row>
     <row r="10" ht="11.1" customHeight="1" spans="1:23">
       <c r="A10" s="20">
@@ -3411,7 +3423,7 @@
       <c r="S10" s="21"/>
       <c r="T10" s="21"/>
       <c r="U10" s="21"/>
-      <c r="V10" s="22"/>
+      <c r="V10" s="19"/>
     </row>
     <row r="11" ht="11.1" customHeight="1" spans="1:23">
       <c r="A11" s="20">
@@ -3437,7 +3449,7 @@
       <c r="S11" s="21"/>
       <c r="T11" s="21"/>
       <c r="U11" s="21"/>
-      <c r="V11" s="22"/>
+      <c r="V11" s="19"/>
     </row>
     <row r="12" ht="11.1" customHeight="1" spans="1:23">
       <c r="A12" s="20">
@@ -3463,7 +3475,7 @@
       <c r="S12" s="21"/>
       <c r="T12" s="21"/>
       <c r="U12" s="21"/>
-      <c r="V12" s="22"/>
+      <c r="V12" s="19"/>
     </row>
     <row r="13" ht="11.1" customHeight="1" spans="1:23">
       <c r="A13" s="20">
@@ -3489,7 +3501,7 @@
       <c r="S13" s="21"/>
       <c r="T13" s="21"/>
       <c r="U13" s="21"/>
-      <c r="V13" s="22"/>
+      <c r="V13" s="19"/>
     </row>
     <row r="14" ht="11.1" customHeight="1" spans="1:23">
       <c r="A14" s="20">
@@ -3515,7 +3527,7 @@
       <c r="S14" s="21"/>
       <c r="T14" s="21"/>
       <c r="U14" s="21"/>
-      <c r="V14" s="22"/>
+      <c r="V14" s="19"/>
     </row>
     <row r="15" ht="11.1" customHeight="1" spans="1:23">
       <c r="A15" s="20">
@@ -3541,7 +3553,7 @@
       <c r="S15" s="21"/>
       <c r="T15" s="21"/>
       <c r="U15" s="21"/>
-      <c r="V15" s="22"/>
+      <c r="V15" s="19"/>
     </row>
     <row r="16" ht="11.1" customHeight="1" spans="1:23">
       <c r="A16" s="20">
@@ -3567,7 +3579,7 @@
       <c r="S16" s="21"/>
       <c r="T16" s="21"/>
       <c r="U16" s="21"/>
-      <c r="V16" s="22"/>
+      <c r="V16" s="19"/>
     </row>
     <row r="17" ht="11.1" customHeight="1" spans="1:22">
       <c r="A17" s="20">
@@ -3593,7 +3605,7 @@
       <c r="S17" s="21"/>
       <c r="T17" s="21"/>
       <c r="U17" s="21"/>
-      <c r="V17" s="22"/>
+      <c r="V17" s="19"/>
     </row>
     <row r="18" ht="11.1" customHeight="1" spans="1:22">
       <c r="A18" s="20">
@@ -3619,7 +3631,7 @@
       <c r="S18" s="21"/>
       <c r="T18" s="21"/>
       <c r="U18" s="21"/>
-      <c r="V18" s="22"/>
+      <c r="V18" s="19"/>
     </row>
     <row r="19" ht="11.1" customHeight="1" spans="1:22">
       <c r="A19" s="20">
@@ -3645,7 +3657,7 @@
       <c r="S19" s="21"/>
       <c r="T19" s="21"/>
       <c r="U19" s="21"/>
-      <c r="V19" s="22"/>
+      <c r="V19" s="19"/>
     </row>
     <row r="20" ht="11.1" customHeight="1" spans="1:22">
       <c r="A20" s="20">
@@ -3671,13 +3683,13 @@
       <c r="S20" s="21"/>
       <c r="T20" s="21"/>
       <c r="U20" s="21"/>
-      <c r="V20" s="22"/>
+      <c r="V20" s="19"/>
     </row>
     <row r="21" ht="11.1" customHeight="1" spans="1:22">
       <c r="A21" s="20">
         <v>14</v>
       </c>
-      <c r="B21" s="23"/>
+      <c r="B21" s="22"/>
       <c r="C21" s="21"/>
       <c r="D21" s="21"/>
       <c r="E21" s="21"/>
@@ -3690,14 +3702,14 @@
       <c r="L21" s="21"/>
       <c r="M21" s="21"/>
       <c r="N21" s="21"/>
-      <c r="O21" s="21"/>
+      <c r="O21" s="23"/>
       <c r="P21" s="21"/>
       <c r="Q21" s="21"/>
       <c r="R21" s="21"/>
       <c r="S21" s="21"/>
       <c r="T21" s="21"/>
       <c r="U21" s="21"/>
-      <c r="V21" s="22"/>
+      <c r="V21" s="19"/>
     </row>
     <row r="22" ht="11.1" customHeight="1" spans="1:22">
       <c r="A22" s="20">
@@ -3723,7 +3735,7 @@
       <c r="S22" s="21"/>
       <c r="T22" s="21"/>
       <c r="U22" s="21"/>
-      <c r="V22" s="22"/>
+      <c r="V22" s="19"/>
     </row>
     <row r="23" ht="11.1" customHeight="1" spans="1:22">
       <c r="A23" s="20">
@@ -3749,7 +3761,7 @@
       <c r="S23" s="21"/>
       <c r="T23" s="21"/>
       <c r="U23" s="21"/>
-      <c r="V23" s="22"/>
+      <c r="V23" s="19"/>
     </row>
     <row r="24" ht="11.1" customHeight="1" spans="1:22">
       <c r="A24" s="20">
@@ -3775,7 +3787,7 @@
       <c r="S24" s="21"/>
       <c r="T24" s="21"/>
       <c r="U24" s="21"/>
-      <c r="V24" s="22"/>
+      <c r="V24" s="19"/>
     </row>
     <row r="25" ht="11.1" customHeight="1" spans="1:22">
       <c r="A25" s="20">
@@ -3801,7 +3813,7 @@
       <c r="S25" s="21"/>
       <c r="T25" s="21"/>
       <c r="U25" s="21"/>
-      <c r="V25" s="22"/>
+      <c r="V25" s="19"/>
     </row>
     <row r="26" ht="11.1" customHeight="1" spans="1:22">
       <c r="A26" s="20">
@@ -3827,7 +3839,7 @@
       <c r="S26" s="21"/>
       <c r="T26" s="21"/>
       <c r="U26" s="21"/>
-      <c r="V26" s="22"/>
+      <c r="V26" s="19"/>
     </row>
     <row r="27" ht="11.1" customHeight="1" spans="1:22">
       <c r="A27" s="20">
@@ -3853,7 +3865,7 @@
       <c r="S27" s="21"/>
       <c r="T27" s="21"/>
       <c r="U27" s="21"/>
-      <c r="V27" s="22"/>
+      <c r="V27" s="19"/>
     </row>
     <row r="28" ht="11.1" customHeight="1" spans="1:22">
       <c r="A28" s="20">
@@ -3879,7 +3891,7 @@
       <c r="S28" s="21"/>
       <c r="T28" s="21"/>
       <c r="U28" s="21"/>
-      <c r="V28" s="22"/>
+      <c r="V28" s="19"/>
     </row>
     <row r="29" ht="11.1" customHeight="1" spans="1:22">
       <c r="A29" s="20">
@@ -3905,7 +3917,7 @@
       <c r="S29" s="21"/>
       <c r="T29" s="21"/>
       <c r="U29" s="21"/>
-      <c r="V29" s="22"/>
+      <c r="V29" s="19"/>
     </row>
     <row r="30" ht="11.1" customHeight="1" spans="1:22">
       <c r="A30" s="20">
@@ -3931,7 +3943,7 @@
       <c r="S30" s="21"/>
       <c r="T30" s="21"/>
       <c r="U30" s="21"/>
-      <c r="V30" s="22"/>
+      <c r="V30" s="19"/>
     </row>
     <row r="31" ht="11.1" customHeight="1" spans="1:22">
       <c r="A31" s="20">
@@ -3957,7 +3969,7 @@
       <c r="S31" s="21"/>
       <c r="T31" s="21"/>
       <c r="U31" s="21"/>
-      <c r="V31" s="22"/>
+      <c r="V31" s="19"/>
     </row>
     <row r="32" ht="11.1" customHeight="1" spans="1:22">
       <c r="A32" s="20">
@@ -3983,7 +3995,7 @@
       <c r="S32" s="21"/>
       <c r="T32" s="21"/>
       <c r="U32" s="21"/>
-      <c r="V32" s="22"/>
+      <c r="V32" s="19"/>
     </row>
     <row r="33" ht="11.1" customHeight="1" spans="1:23">
       <c r="A33" s="20">
@@ -4009,7 +4021,7 @@
       <c r="S33" s="21"/>
       <c r="T33" s="21"/>
       <c r="U33" s="21"/>
-      <c r="V33" s="22"/>
+      <c r="V33" s="19"/>
     </row>
     <row r="34" ht="11.1" customHeight="1" spans="1:23">
       <c r="A34" s="20">
@@ -4035,7 +4047,7 @@
       <c r="S34" s="21"/>
       <c r="T34" s="21"/>
       <c r="U34" s="21"/>
-      <c r="V34" s="22"/>
+      <c r="V34" s="19"/>
     </row>
     <row r="35" ht="11.1" customHeight="1" spans="1:23">
       <c r="A35" s="20">
@@ -4061,7 +4073,7 @@
       <c r="S35" s="21"/>
       <c r="T35" s="21"/>
       <c r="U35" s="21"/>
-      <c r="V35" s="22"/>
+      <c r="V35" s="19"/>
     </row>
     <row r="36" ht="11.1" customHeight="1" spans="1:23">
       <c r="A36" s="20">
@@ -4087,7 +4099,7 @@
       <c r="S36" s="21"/>
       <c r="T36" s="21"/>
       <c r="U36" s="21"/>
-      <c r="V36" s="22"/>
+      <c r="V36" s="19"/>
     </row>
     <row r="37" ht="11.1" customHeight="1" spans="1:23">
       <c r="A37" s="20">
@@ -4113,7 +4125,7 @@
       <c r="S37" s="21"/>
       <c r="T37" s="21"/>
       <c r="U37" s="21"/>
-      <c r="V37" s="22"/>
+      <c r="V37" s="19"/>
     </row>
     <row r="38" ht="11.1" customHeight="1" spans="1:23">
       <c r="A38" s="20">
@@ -4365,7 +4377,7 @@
       <c r="S43" s="21"/>
       <c r="T43" s="21"/>
       <c r="U43" s="21"/>
-      <c r="V43" s="22"/>
+      <c r="V43" s="19"/>
     </row>
     <row r="44" ht="11.1" customHeight="1" spans="1:23">
       <c r="A44" s="20">
@@ -4391,7 +4403,7 @@
       <c r="S44" s="21"/>
       <c r="T44" s="21"/>
       <c r="U44" s="21"/>
-      <c r="V44" s="22"/>
+      <c r="V44" s="19"/>
     </row>
     <row r="45" ht="11.1" customHeight="1" spans="1:23">
       <c r="A45" s="20">
@@ -4417,7 +4429,7 @@
       <c r="S45" s="21"/>
       <c r="T45" s="21"/>
       <c r="U45" s="21"/>
-      <c r="V45" s="22"/>
+      <c r="V45" s="19"/>
     </row>
     <row r="46" ht="11.1" customHeight="1" spans="1:23">
       <c r="A46" s="20">
@@ -4443,7 +4455,7 @@
       <c r="S46" s="21"/>
       <c r="T46" s="21"/>
       <c r="U46" s="21"/>
-      <c r="V46" s="22"/>
+      <c r="V46" s="19"/>
     </row>
     <row r="47" ht="11.1" customHeight="1" spans="1:23">
       <c r="A47" s="20">
@@ -4469,7 +4481,7 @@
       <c r="S47" s="21"/>
       <c r="T47" s="21"/>
       <c r="U47" s="21"/>
-      <c r="V47" s="22"/>
+      <c r="V47" s="19"/>
     </row>
     <row r="48" ht="11.1" customHeight="1" spans="1:23">
       <c r="A48" s="20">
@@ -4495,7 +4507,7 @@
       <c r="S48" s="21"/>
       <c r="T48" s="21"/>
       <c r="U48" s="21"/>
-      <c r="V48" s="22"/>
+      <c r="V48" s="19"/>
     </row>
     <row r="49" ht="11.1" customHeight="1" spans="1:22">
       <c r="A49" s="20">
@@ -4521,7 +4533,7 @@
       <c r="S49" s="21"/>
       <c r="T49" s="21"/>
       <c r="U49" s="21"/>
-      <c r="V49" s="22"/>
+      <c r="V49" s="19"/>
     </row>
     <row r="50" ht="11.1" customHeight="1" spans="1:22">
       <c r="A50" s="20">
@@ -4547,7 +4559,7 @@
       <c r="S50" s="21"/>
       <c r="T50" s="21"/>
       <c r="U50" s="21"/>
-      <c r="V50" s="22"/>
+      <c r="V50" s="19"/>
     </row>
     <row r="51" ht="11.1" customHeight="1" spans="1:22">
       <c r="A51" s="20">
@@ -4573,7 +4585,7 @@
       <c r="S51" s="21"/>
       <c r="T51" s="21"/>
       <c r="U51" s="21"/>
-      <c r="V51" s="22"/>
+      <c r="V51" s="19"/>
     </row>
     <row r="52" ht="11.1" customHeight="1" spans="1:22">
       <c r="A52" s="20">
@@ -4599,7 +4611,7 @@
       <c r="S52" s="21"/>
       <c r="T52" s="21"/>
       <c r="U52" s="21"/>
-      <c r="V52" s="22"/>
+      <c r="V52" s="19"/>
     </row>
     <row r="53" ht="11.1" customHeight="1" spans="1:22">
       <c r="A53" s="20">
@@ -4625,7 +4637,7 @@
       <c r="S53" s="21"/>
       <c r="T53" s="21"/>
       <c r="U53" s="21"/>
-      <c r="V53" s="22"/>
+      <c r="V53" s="19"/>
     </row>
     <row r="54" ht="11.1" customHeight="1" spans="1:22">
       <c r="A54" s="20">
@@ -4651,7 +4663,7 @@
       <c r="S54" s="21"/>
       <c r="T54" s="21"/>
       <c r="U54" s="21"/>
-      <c r="V54" s="22"/>
+      <c r="V54" s="19"/>
     </row>
     <row r="55" ht="11.1" customHeight="1" spans="1:22">
       <c r="A55" s="20">
@@ -4677,7 +4689,7 @@
       <c r="S55" s="21"/>
       <c r="T55" s="21"/>
       <c r="U55" s="21"/>
-      <c r="V55" s="22"/>
+      <c r="V55" s="19"/>
     </row>
     <row r="56" ht="11.1" customHeight="1" spans="1:22">
       <c r="A56" s="20">
@@ -4702,7 +4714,7 @@
       <c r="S56" s="21"/>
       <c r="T56" s="21"/>
       <c r="U56" s="21"/>
-      <c r="V56" s="22"/>
+      <c r="V56" s="19"/>
     </row>
     <row r="57" ht="11.1" customHeight="1" spans="1:22">
       <c r="A57" s="20">
@@ -4728,7 +4740,7 @@
       <c r="S57" s="21"/>
       <c r="T57" s="21"/>
       <c r="U57" s="21"/>
-      <c r="V57" s="22"/>
+      <c r="V57" s="19"/>
     </row>
     <row r="58" ht="11.1" customHeight="1" spans="1:22">
       <c r="A58" s="20">
@@ -4754,7 +4766,7 @@
       <c r="S58" s="21"/>
       <c r="T58" s="21"/>
       <c r="U58" s="21"/>
-      <c r="V58" s="22"/>
+      <c r="V58" s="19"/>
     </row>
     <row r="59" ht="11.1" customHeight="1" spans="1:22">
       <c r="A59" s="20">
@@ -4780,7 +4792,7 @@
       <c r="S59" s="21"/>
       <c r="T59" s="21"/>
       <c r="U59" s="21"/>
-      <c r="V59" s="22"/>
+      <c r="V59" s="19"/>
     </row>
     <row r="60" ht="11.1" customHeight="1" spans="1:22">
       <c r="A60" s="20">
@@ -4806,7 +4818,7 @@
       <c r="S60" s="21"/>
       <c r="T60" s="21"/>
       <c r="U60" s="21"/>
-      <c r="V60" s="22"/>
+      <c r="V60" s="19"/>
     </row>
     <row r="61" ht="11.1" customHeight="1" spans="1:22">
       <c r="A61" s="20">
@@ -4832,7 +4844,7 @@
       <c r="S61" s="21"/>
       <c r="T61" s="21"/>
       <c r="U61" s="21"/>
-      <c r="V61" s="22"/>
+      <c r="V61" s="19"/>
     </row>
     <row r="62" ht="11.1" customHeight="1" spans="1:22">
       <c r="A62" s="20">
@@ -4858,7 +4870,7 @@
       <c r="S62" s="21"/>
       <c r="T62" s="21"/>
       <c r="U62" s="21"/>
-      <c r="V62" s="22"/>
+      <c r="V62" s="19"/>
     </row>
     <row r="63" ht="11.1" customHeight="1" spans="1:22">
       <c r="A63" s="20">
@@ -4884,7 +4896,7 @@
       <c r="S63" s="21"/>
       <c r="T63" s="21"/>
       <c r="U63" s="21"/>
-      <c r="V63" s="22"/>
+      <c r="V63" s="19"/>
     </row>
     <row r="64" ht="11.1" customHeight="1" spans="1:22">
       <c r="A64" s="20">
@@ -4910,7 +4922,7 @@
       <c r="S64" s="21"/>
       <c r="T64" s="21"/>
       <c r="U64" s="21"/>
-      <c r="V64" s="22"/>
+      <c r="V64" s="19"/>
     </row>
     <row r="65" ht="11.1" customHeight="1" spans="1:25">
       <c r="A65" s="20">
@@ -4936,7 +4948,7 @@
       <c r="S65" s="21"/>
       <c r="T65" s="21"/>
       <c r="U65" s="21"/>
-      <c r="V65" s="22"/>
+      <c r="V65" s="19"/>
     </row>
     <row r="66" ht="11.1" customHeight="1" spans="1:25">
       <c r="A66" s="20">
@@ -4962,7 +4974,7 @@
       <c r="S66" s="21"/>
       <c r="T66" s="21"/>
       <c r="U66" s="21"/>
-      <c r="V66" s="22"/>
+      <c r="V66" s="19"/>
     </row>
     <row r="67" ht="11.1" customHeight="1" spans="1:25">
       <c r="A67" s="20">
@@ -4988,7 +5000,7 @@
       <c r="S67" s="21"/>
       <c r="T67" s="21"/>
       <c r="U67" s="21"/>
-      <c r="V67" s="22"/>
+      <c r="V67" s="19"/>
     </row>
     <row r="68" ht="11.1" customHeight="1" spans="1:25">
       <c r="A68" s="20">
@@ -5014,7 +5026,7 @@
       <c r="S68" s="21"/>
       <c r="T68" s="21"/>
       <c r="U68" s="21"/>
-      <c r="V68" s="22"/>
+      <c r="V68" s="19"/>
     </row>
     <row r="69" ht="11.1" customHeight="1" spans="1:25">
       <c r="A69" s="20">
@@ -5040,7 +5052,7 @@
       <c r="S69" s="21"/>
       <c r="T69" s="21"/>
       <c r="U69" s="21"/>
-      <c r="V69" s="22"/>
+      <c r="V69" s="19"/>
     </row>
     <row r="70" ht="11.1" customHeight="1" spans="1:25">
       <c r="A70" s="20">
@@ -5066,7 +5078,7 @@
       <c r="S70" s="21"/>
       <c r="T70" s="21"/>
       <c r="U70" s="21"/>
-      <c r="V70" s="22"/>
+      <c r="V70" s="19"/>
     </row>
     <row r="71" ht="11.1" customHeight="1" spans="1:25">
       <c r="A71" s="20">
@@ -5092,7 +5104,7 @@
       <c r="S71" s="21"/>
       <c r="T71" s="21"/>
       <c r="U71" s="21"/>
-      <c r="V71" s="22"/>
+      <c r="V71" s="19"/>
     </row>
     <row r="72" ht="11.1" customHeight="1" spans="1:25">
       <c r="A72" s="20">
@@ -5118,7 +5130,7 @@
       <c r="S72" s="21"/>
       <c r="T72" s="21"/>
       <c r="U72" s="21"/>
-      <c r="V72" s="22"/>
+      <c r="V72" s="19"/>
     </row>
     <row r="73" ht="11.1" customHeight="1" spans="1:25">
       <c r="A73" s="20">

</xml_diff>